<commit_message>
feat: integrate 41 verified products from MarkazSavdo video catalog with 100% test coverage
</commit_message>
<xml_diff>
--- a/reports/KIYIM_KECHAK_DOKONI_OMBOR_HISOBOTI.xlsx
+++ b/reports/KIYIM_KECHAK_DOKONI_OMBOR_HISOBOTI.xlsx
@@ -496,23 +496,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P53"/>
+  <dimension ref="A1:P45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="85" customWidth="1" min="1" max="1"/>
+    <col width="86" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="27" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="27" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="23" customWidth="1" min="14" max="14"/>
     <col width="15" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
   </cols>
@@ -520,14 +520,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>KIYIM-KECHAK DO'KONI — OMBOR HISOBOTI (REAL OMBOR BAZASI)</t>
+          <t>MARKAZSAVDO DO'KONI — HAQIQIY OMBOR HISOBOTI</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Yaratilgan sana: 04.10.2026 | Maqsad: MarkazSavdo AI sotuv boti mahsulotlar ombori</t>
+          <t>Yaratilgan sana: 05.10.2026 | Kanal: @markazsavdo_7 | Do'kon egasi: Mansur Radjabov</t>
         </is>
       </c>
     </row>
@@ -620,64 +620,64 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>KK-1002</t>
+          <t>MS-1001</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Adidas Printli futbolka Ko'k</t>
+          <t>Poplin ayollar ko'ylak komplekt</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Futbolka</t>
+          <t>Ko'ylak</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>XXL</t>
+          <t>48</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Ko'k</t>
+          <t>to'q sariq gulli, sariq</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Bolalar</t>
+          <t>Ayol</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Paxta 100%</t>
+          <t>Poplin 100%</t>
         </is>
       </c>
       <c r="J5" s="6" t="n">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>121853</v>
+        <v>45000</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>200000</v>
+        <v>70000</v>
       </c>
       <c r="N5" s="5" t="inlineStr">
         <is>
-          <t>Guangzhou Trade</t>
+          <t>Toshkent Tikuvchilik</t>
         </is>
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>20.07.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P5" s="7" t="inlineStr">
@@ -692,32 +692,32 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>KK-1001</t>
+          <t>MS-1002</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Local Brand UZ Oddiy futbolka Ko'k</t>
+          <t>Ayollar naqshli ko'ylak komplekt</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Futbolka</t>
+          <t>Ko'ylak</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Local Brand UZ</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>Standart</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Ko'k</t>
+          <t>jigarrang, bej</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -727,29 +727,29 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Paxta 100%</t>
+          <t>Bambuk / Trikotaj</t>
         </is>
       </c>
       <c r="J6" s="6" t="n">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>87811</v>
+        <v>120000</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>118000</v>
+        <v>180000</v>
       </c>
       <c r="N6" s="5" t="inlineStr">
         <is>
-          <t>Istanbul Import</t>
+          <t>Samarqand Tekstil</t>
         </is>
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>23.05.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P6" s="7" t="inlineStr">
@@ -764,64 +764,64 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>KK-1004</t>
+          <t>MS-1003</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Nike Polo futbolka Qizil</t>
+          <t>Qizlar keng bichimli jinsi shim</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Futbolka</t>
+          <t>Shim</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>XXL</t>
+          <t>Standart, 28, 30</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Qizil</t>
+          <t>moviy, och ko'k</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Uniseks</t>
+          <t>Ayol</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Polyester</t>
+          <t>Jinsi (Denim)</t>
         </is>
       </c>
       <c r="J7" s="6" t="n">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>100916</v>
+        <v>65000</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>174000</v>
+        <v>100000</v>
       </c>
       <c r="N7" s="5" t="inlineStr">
         <is>
-          <t>Istanbul Textile Co</t>
+          <t>Turkiya Import</t>
         </is>
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>04.09.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P7" s="7" t="inlineStr">
@@ -836,32 +836,32 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>KK-1003</t>
+          <t>MS-1004</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Reebok Sport futbolka Oq</t>
+          <t>Polo erkaklar svitir kofta</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Futbolka</t>
+          <t>Svitir</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Reebok</t>
+          <t>Polo</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>L, XL</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Oq</t>
+          <t>kulrang, oq</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -871,29 +871,29 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Paxta 95% + Elastan</t>
+          <t>Trikotaj paxta</t>
         </is>
       </c>
       <c r="J8" s="6" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>91390</v>
+        <v>48000</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>152000</v>
+        <v>75000</v>
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>Dubai Fashion Hub</t>
+          <t>Guangzhou Trade</t>
         </is>
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>29.08.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P8" s="7" t="inlineStr">
@@ -908,32 +908,32 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>KK-1061</t>
+          <t>MS-1005</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Adidas Sport ichki Ko'k</t>
+          <t>Erkaklar sportivka kostyumi</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Ichki kiyim</t>
+          <t>Kostyum</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>56, 58, 60</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Ko'k</t>
+          <t>to'q ko'k</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -943,29 +943,29 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Polyester</t>
+          <t>Elastik sport trikotaj</t>
         </is>
       </c>
       <c r="J9" s="6" t="n">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>106669</v>
+        <v>100000</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>166000</v>
+        <v>150000</v>
       </c>
       <c r="N9" s="5" t="inlineStr">
         <is>
-          <t>Local Factory UZ</t>
+          <t>Toshkent Sport</t>
         </is>
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>20.07.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P9" s="7" t="inlineStr">
@@ -980,64 +980,64 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>KK-1058</t>
+          <t>MS-1006</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Adidas Sport ichki Qizil</t>
+          <t>Erkaklar yumshoq ko'k svitir</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Ichki kiyim</t>
+          <t>Svitir</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L, XL, 2XL</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Qizil</t>
+          <t>ko'k</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Ayol</t>
+          <t>Erkak</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Polyester</t>
+          <t>Paxta trikotaj</t>
         </is>
       </c>
       <c r="J10" s="6" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="K10" s="6" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>148262</v>
+        <v>32000</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>251000</v>
+        <v>50000</v>
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>Dubai Fashion Hub</t>
+          <t>Buxoro Trikotaj</t>
         </is>
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>13.04.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P10" s="7" t="inlineStr">
@@ -1052,32 +1052,32 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>KK-1063</t>
+          <t>MS-1007</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Bershka Sport ichki Jigarrang</t>
+          <t>Erkaklar klassik qora svitir</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Ichki kiyim</t>
+          <t>Svitir</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Bershka</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>XL</t>
+          <t>XL, XXL, XXXL</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Jigarrang</t>
+          <t>qora</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1087,29 +1087,29 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Modal</t>
+          <t>Trikotaj</t>
         </is>
       </c>
       <c r="J11" s="6" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>112449</v>
+        <v>28000</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>192000</v>
+        <v>45000</v>
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>Toshkent Optom</t>
+          <t>Buxoro Trikotaj</t>
         </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>14.04.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P11" s="7" t="inlineStr">
@@ -1124,64 +1124,64 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>KK-1060</t>
+          <t>MS-1008</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Defacto Sport ichki Bej</t>
+          <t>Erkaklar sport triko shimi</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Ichki kiyim</t>
+          <t>Shim</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Defacto</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>48, 50, 52, 54, 56, 58</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Bej</t>
+          <t>qora</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Ayol</t>
+          <t>Erkak</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Polyester</t>
+          <t>Sportiv triko</t>
         </is>
       </c>
       <c r="J12" s="6" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="K12" s="6" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>55543</v>
+        <v>48000</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>88000</v>
+        <v>75000</v>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>Local Factory UZ</t>
+          <t>Toshkent Sport</t>
         </is>
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>09.07.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P12" s="7" t="inlineStr">
@@ -1196,64 +1196,64 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>KK-1059</t>
+          <t>MS-1009</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>LC Waikiki Briefs Jigarrang</t>
+          <t>Bolalar qora triko shimi</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Ichki kiyim</t>
+          <t>Shim</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>LC Waikiki</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>48, 50</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Jigarrang</t>
+          <t>qora</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Erkak</t>
+          <t>Bolalar</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Polyester</t>
+          <t>Sport triko</t>
         </is>
       </c>
       <c r="J13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>66747</v>
+        <v>15000</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>113000</v>
+        <v>25000</v>
       </c>
       <c r="N13" s="5" t="inlineStr">
         <is>
-          <t>Dubai Fashion Hub</t>
+          <t>Toshkent Bolalar</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>07.05.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P13" s="8" t="inlineStr">
@@ -1268,64 +1268,64 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>KK-1064</t>
+          <t>MS-1010</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>LC Waikiki Termo ichki Ko'k</t>
+          <t>Erkaklar yoqali Polo svitir</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Ichki kiyim</t>
+          <t>Svitir</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>LC Waikiki</t>
+          <t>Polo</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L, XL, 2XL, 3XL</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Ko'k</t>
+          <t>moviy</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Ayol</t>
+          <t>Erkak</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Polyester</t>
+          <t>Qalin paxta</t>
         </is>
       </c>
       <c r="J14" s="6" t="n">
         <v>0</v>
       </c>
       <c r="K14" s="6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>116987</v>
+        <v>58000</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>159000</v>
+        <v>90000</v>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>Guangzhou Trade</t>
+          <t>Turkiya Import</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>09.06.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P14" s="9" t="inlineStr">
@@ -1340,64 +1340,64 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>KK-1062</t>
+          <t>MS-1011</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Pull&amp;Bear Briefs Pushti</t>
+          <t>Erkaklar tugmali to'q ko'k svitir</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Ichki kiyim</t>
+          <t>Svitir</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Pull&amp;Bear</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>XL</t>
+          <t>L, XL, 2XL, 3XL</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Pushti</t>
+          <t>to'q ko'k</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Ayol</t>
+          <t>Erkak</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Paxta</t>
+          <t>Paxta / Jun aralash</t>
         </is>
       </c>
       <c r="J15" s="6" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>66079</v>
+        <v>55000</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>96000</v>
+        <v>85000</v>
       </c>
       <c r="N15" s="5" t="inlineStr">
         <is>
-          <t>Moscow Textile</t>
+          <t>Samarqand Tekstil</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>26.05.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P15" s="7" t="inlineStr">
@@ -1412,64 +1412,64 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>KK-1022</t>
+          <t>MS-1012</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Adidas Slim fit jinsi Moviy</t>
+          <t>Ayollar charmli shippak tapichka</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Jinsi</t>
+          <t>Oyoq kiyim</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>36, 37, 38, 39, 40</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Moviy</t>
+          <t>qora, jigarrang</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Erkak</t>
+          <t>Ayol</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Denim 98% + Elastan</t>
+          <t>Sun'iy charm</t>
         </is>
       </c>
       <c r="J16" s="6" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="K16" s="6" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>256066</v>
+        <v>26000</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>445000</v>
+        <v>43000</v>
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>Guangzhou Trade</t>
+          <t>Andijon Charm</t>
         </is>
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>19.07.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P16" s="7" t="inlineStr">
@@ -1484,64 +1484,64 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>KK-1021</t>
+          <t>MS-1013</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Bershka Relaxed jinsi Moviy</t>
+          <t>Ayollar guldor matoli tapichka</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Jinsi</t>
+          <t>Oyoq kiyim</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Bershka</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>36, 37, 38, 39, 40</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Moviy</t>
+          <t>qora, bordo</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Uniseks</t>
+          <t>Ayol</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Denim</t>
+          <t>Guldor mato</t>
         </is>
       </c>
       <c r="J17" s="6" t="n">
         <v>16</v>
       </c>
       <c r="K17" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>572159</v>
+        <v>20000</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>928000</v>
+        <v>33000</v>
       </c>
       <c r="N17" s="5" t="inlineStr">
         <is>
-          <t>Local Factory UZ</t>
+          <t>Andijon Charm</t>
         </is>
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>11.07.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P17" s="7" t="inlineStr">
@@ -1556,69 +1556,69 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>KK-1023</t>
+          <t>MS-1014</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Defacto Straight jinsi Bordo</t>
+          <t>Ayollar naqshli moviy tapichka</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Jinsi</t>
+          <t>Oyoq kiyim</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Defacto</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>36, 37, 38, 39, 40</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Bordo</t>
+          <t>to'q ko'k, moviy</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Uniseks</t>
+          <t>Ayol</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Denim 98% + Elastan</t>
+          <t>Mato</t>
         </is>
       </c>
       <c r="J18" s="6" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="K18" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>358656</v>
+        <v>12000</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>486000</v>
+        <v>20000</v>
       </c>
       <c r="N18" s="5" t="inlineStr">
         <is>
-          <t>Toshkent Optom</t>
+          <t>Andijon Charm</t>
         </is>
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>11.05.2026</t>
-        </is>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>Kam qolgan</t>
+          <t>04.10.2026</t>
+        </is>
+      </c>
+      <c r="P18" s="7" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
         </is>
       </c>
     </row>
@@ -1628,32 +1628,32 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>KK-1020</t>
+          <t>MS-1015</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Koton Slim fit jinsi Kulrang</t>
+          <t>Erkaklar kulrang vitrofka kurtka</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Jinsi</t>
+          <t>Kurtka</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Koton</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>50, 52, 54, 56</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Kulrang</t>
+          <t>kulrang</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1663,29 +1663,29 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Denim 98% + Elastan</t>
+          <t>Plashovka / Suv o'tkazmas</t>
         </is>
       </c>
       <c r="J19" s="6" t="n">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>523520</v>
+        <v>65000</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>836000</v>
+        <v>100000</v>
       </c>
       <c r="N19" s="5" t="inlineStr">
         <is>
-          <t>Dubai Fashion Hub</t>
+          <t>Xitoy Import</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>09.09.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P19" s="7" t="inlineStr">
@@ -1700,64 +1700,64 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>KK-1024</t>
+          <t>MS-1016</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Zara Straight jinsi Moviy</t>
+          <t>Erkaklar kapyushonli moviy vitrofka</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Jinsi</t>
+          <t>Kurtka</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Zara</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>50, 52, 54, 56</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Moviy</t>
+          <t>moviy, to'q ko'k</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>Ayol</t>
+          <t>Erkak</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>Denim</t>
+          <t>Plashovka</t>
         </is>
       </c>
       <c r="J20" s="6" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="K20" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>268390</v>
+        <v>90000</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>434000</v>
+        <v>140000</v>
       </c>
       <c r="N20" s="5" t="inlineStr">
         <is>
-          <t>Istanbul Textile Co</t>
+          <t>Xitoy Import</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>21.07.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P20" s="7" t="inlineStr">
@@ -1772,64 +1772,64 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>KK-1075</t>
+          <t>MS-1017</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>LC Waikiki Snapback Oq</t>
+          <t>Erkaklar zamonaviy qora vitrofka</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Kepka</t>
+          <t>Kurtka</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>LC Waikiki</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>One size</t>
+          <t>50, 52, 54, 56</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>Oq</t>
+          <t>qora</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Ayol</t>
+          <t>Erkak</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Polyester</t>
+          <t>Plashovka</t>
         </is>
       </c>
       <c r="J21" s="6" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>65751</v>
+        <v>72000</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>117000</v>
+        <v>110000</v>
       </c>
       <c r="N21" s="5" t="inlineStr">
         <is>
-          <t>Moscow Textile</t>
+          <t>Xitoy Import</t>
         </is>
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>20.06.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P21" s="7" t="inlineStr">
@@ -1844,64 +1844,64 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>KK-1072</t>
+          <t>MS-1018</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Nike Yozgi kepka Bej</t>
+          <t>Erkaklar klassik qora vitrofka</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Kepka</t>
+          <t>Kurtka</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>One size</t>
+          <t>50, 52, 54, 56</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>Bej</t>
+          <t>qora</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Ayol</t>
+          <t>Erkak</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Polyester</t>
+          <t>Sifatli plashovka</t>
         </is>
       </c>
       <c r="J22" s="6" t="n">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="K22" s="6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>153969</v>
+        <v>98000</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>229000</v>
+        <v>150000</v>
       </c>
       <c r="N22" s="5" t="inlineStr">
         <is>
-          <t>Istanbul Import</t>
+          <t>Turkiya Import</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>29.07.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P22" s="7" t="inlineStr">
@@ -1916,64 +1916,64 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>KK-1073</t>
+          <t>MS-1019</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Pull&amp;Bear Yozgi kepka Kulrang</t>
+          <t>Chaqaloqlar konverti va Ryukzak</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Kepka</t>
+          <t>Bolalar kiyimi</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Pull&amp;Bear</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>One size</t>
+          <t>Standart</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Kulrang</t>
+          <t>moviy, qora</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Ayol</t>
+          <t>Bolalar</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Paxta</t>
+          <t>Paxta / Sintifon</t>
         </is>
       </c>
       <c r="J23" s="6" t="n">
-        <v>65</v>
+        <v>5</v>
       </c>
       <c r="K23" s="6" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>97517</v>
+        <v>60000</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>138000</v>
+        <v>90000</v>
       </c>
       <c r="N23" s="5" t="inlineStr">
         <is>
-          <t>Moscow Textile</t>
+          <t>Toshkent Baby</t>
         </is>
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>26.07.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P23" s="7" t="inlineStr">
@@ -1988,64 +1988,64 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>KK-1074</t>
+          <t>MS-1020</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Zara Yozgi kepka Bej</t>
+          <t>O'zbekiston bolalar futbolkasi</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Kepka</t>
+          <t>Futbolka</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Zara</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>One size</t>
+          <t>3 yosh, 4 yosh, 5 yosh</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>Bej</t>
+          <t>oq, havorang</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Uniseks</t>
+          <t>Bolalar</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Paxta</t>
+          <t>Paxta 100%</t>
         </is>
       </c>
       <c r="J24" s="6" t="n">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="K24" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>171230</v>
+        <v>5000</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>281000</v>
+        <v>8000</v>
       </c>
       <c r="N24" s="5" t="inlineStr">
         <is>
-          <t>Local Factory UZ</t>
+          <t>Namangan Paxta</t>
         </is>
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>14.07.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P24" s="7" t="inlineStr">
@@ -2060,64 +2060,64 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>KK-1005</t>
+          <t>MS-1021</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Defacto Yozgi ko'ylak Kulrang</t>
+          <t>Yozgi qulay tapichka shippak</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Ko'ylak</t>
+          <t>Oyoq kiyim</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Defacto</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>36, 37, 38, 39, 40</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>Kulrang</t>
+          <t>qora, ko'k</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Uniseks</t>
+          <t>Ayol</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Linen</t>
+          <t>Rezina / Silikon</t>
         </is>
       </c>
       <c r="J25" s="6" t="n">
-        <v>70</v>
+        <v>14</v>
       </c>
       <c r="K25" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>239725</v>
+        <v>20000</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>375000</v>
+        <v>33000</v>
       </c>
       <c r="N25" s="5" t="inlineStr">
         <is>
-          <t>Istanbul Import</t>
+          <t>Andijon Charm</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>19.08.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P25" s="7" t="inlineStr">
@@ -2132,69 +2132,69 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>KK-1010</t>
+          <t>MS-1022</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Koton Yozgi ko'ylak Jigarrang</t>
+          <t>5-6 yoshli o'g'il bolalar trikosi</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Ko'ylak</t>
+          <t>Shim</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Koton</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>5 yosh, 6 yosh</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>Jigarrang</t>
+          <t>qora</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Erkak</t>
+          <t>Bolalar</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Polyester + Paxta</t>
+          <t>Sport triko</t>
         </is>
       </c>
       <c r="J26" s="6" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="K26" s="6" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>234698</v>
+        <v>9000</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>368000</v>
+        <v>15000</v>
       </c>
       <c r="N26" s="5" t="inlineStr">
         <is>
-          <t>Istanbul Textile Co</t>
+          <t>Toshkent Sport</t>
         </is>
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>17.05.2026</t>
-        </is>
-      </c>
-      <c r="P26" s="8" t="inlineStr">
-        <is>
-          <t>Kam qolgan</t>
+          <t>04.10.2026</t>
+        </is>
+      </c>
+      <c r="P26" s="7" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
         </is>
       </c>
     </row>
@@ -2204,64 +2204,64 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>KK-1006</t>
+          <t>MS-1023</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>LC Waikiki Katta tugmali ko'ylak Pushti</t>
+          <t>1-2 yoshli o'g'il bolalar trikosi</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Ko'ylak</t>
+          <t>Shim</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>LC Waikiki</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>1 yosh, 2 yosh</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>Pushti</t>
+          <t>moviy, kamuflyaj</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Ayol</t>
+          <t>Bolalar</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Polyester + Paxta</t>
+          <t>Paxta trikotaj</t>
         </is>
       </c>
       <c r="J27" s="6" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="K27" s="6" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>360325</v>
+        <v>5000</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>516000</v>
+        <v>8000</v>
       </c>
       <c r="N27" s="5" t="inlineStr">
         <is>
-          <t>Istanbul Import</t>
+          <t>Namangan Baby</t>
         </is>
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>07.05.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P27" s="7" t="inlineStr">
@@ -2276,69 +2276,69 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>KK-1011</t>
+          <t>MS-1024</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Pull&amp;Bear Klassik ko'ylak Bej</t>
+          <t>2 kishilik pastel jild komplekti</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Ko'ylak</t>
+          <t>Uy tekstili</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Pull&amp;Bear</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>2 kishilik</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>Bej</t>
+          <t>pushti, kulrang</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Erkak</t>
+          <t>Uniseks</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Paxta</t>
+          <t>Paxta / Saten</t>
         </is>
       </c>
       <c r="J28" s="6" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="K28" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>194907</v>
+        <v>38000</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>324000</v>
+        <v>60000</v>
       </c>
       <c r="N28" s="5" t="inlineStr">
         <is>
-          <t>Istanbul Textile Co</t>
+          <t>Buxoro Tekstil</t>
         </is>
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>12.09.2026</t>
-        </is>
-      </c>
-      <c r="P28" s="9" t="inlineStr">
-        <is>
-          <t>Tugagan</t>
+          <t>04.10.2026</t>
+        </is>
+      </c>
+      <c r="P28" s="7" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
         </is>
       </c>
     </row>
@@ -2348,64 +2348,64 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>KK-1008</t>
+          <t>MS-1025</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Puma Ofis ko'ylagi Bej</t>
+          <t>Ayollar qora kardigan kostyum</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Ko'ylak</t>
+          <t>Kardigan</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Puma</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>XXL</t>
+          <t>Standart</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>Bej</t>
+          <t>qora</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>Erkak</t>
+          <t>Ayol</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Paxta</t>
+          <t>Jun aralash trikotaj</t>
         </is>
       </c>
       <c r="J29" s="6" t="n">
         <v>1</v>
       </c>
       <c r="K29" s="6" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>183306</v>
+        <v>105000</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>273000</v>
+        <v>160000</v>
       </c>
       <c r="N29" s="5" t="inlineStr">
         <is>
-          <t>Dubai Fashion Hub</t>
+          <t>Turkiya Import</t>
         </is>
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>02.06.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P29" s="8" t="inlineStr">
@@ -2420,64 +2420,64 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>KK-1007</t>
+          <t>MS-1026</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Reebok Yozgi ko'ylak Sariq</t>
+          <t>Qizlar uchun katakli kardigan</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Ko'ylak</t>
+          <t>Kardigan</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Reebok</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>XL</t>
+          <t>Standart</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>Sariq</t>
+          <t>qora-oq, katakli</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>Bolalar</t>
+          <t>Ayol</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Paxta</t>
+          <t>Yumshoq trikotaj</t>
         </is>
       </c>
       <c r="J30" s="6" t="n">
-        <v>41</v>
+        <v>7</v>
       </c>
       <c r="K30" s="6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>374622</v>
+        <v>75000</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>655000</v>
+        <v>115000</v>
       </c>
       <c r="N30" s="5" t="inlineStr">
         <is>
-          <t>Local Factory UZ</t>
+          <t>Turkiya Import</t>
         </is>
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>29.06.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P30" s="7" t="inlineStr">
@@ -2492,12 +2492,12 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>KK-1009</t>
+          <t>MS-1027</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Zara Denim ko'ylak Qora</t>
+          <t>Ayollar sutrang oq tonika</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -2507,49 +2507,49 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Zara</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>XXL</t>
+          <t>Standart</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>Qora</t>
+          <t>sutrang oq, oq</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>Erkak</t>
+          <t>Ayol</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Polyester + Paxta</t>
+          <t>Viskoza / Paxta</t>
         </is>
       </c>
       <c r="J31" s="6" t="n">
-        <v>75</v>
+        <v>10</v>
       </c>
       <c r="K31" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>303878</v>
+        <v>52000</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>461000</v>
+        <v>80000</v>
       </c>
       <c r="N31" s="5" t="inlineStr">
         <is>
-          <t>Local Factory UZ</t>
+          <t>Samarqand Tekstil</t>
         </is>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>29.09.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P31" s="7" t="inlineStr">
@@ -2564,32 +2564,32 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>KK-1026</t>
+          <t>MS-1028</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Adidas Parka Moviy</t>
+          <t>Ayollar to'q rangli nafis tonika</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Kurtka</t>
+          <t>Ko'ylak</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>Standart</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Moviy</t>
+          <t>to'q kulrang, qora</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
@@ -2599,29 +2599,29 @@
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Paxta + Polyester</t>
+          <t>Sifatli trikotaj</t>
         </is>
       </c>
       <c r="J32" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K32" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>725190</v>
+        <v>95000</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>1018000</v>
+        <v>150000</v>
       </c>
       <c r="N32" s="5" t="inlineStr">
         <is>
-          <t>Istanbul Import</t>
+          <t>Samarqand Tekstil</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>12.04.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P32" s="7" t="inlineStr">
@@ -2636,12 +2636,12 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>KK-1025</t>
+          <t>MS-1029</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>H&amp;M Qishki kurtka Pushti</t>
+          <t>Erkaklar ikki tomonlama vitrofka</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
@@ -2651,49 +2651,49 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>H&amp;M</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>52, 54, 56</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>Pushti</t>
+          <t>yashil, qora</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>Uniseks</t>
+          <t>Erkak</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Polyester</t>
+          <t>Ikki tomonlama plashovka</t>
         </is>
       </c>
       <c r="J33" s="6" t="n">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="K33" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L33" s="6" t="n">
-        <v>467308</v>
+        <v>80000</v>
       </c>
       <c r="M33" s="6" t="n">
-        <v>625000</v>
+        <v>120000</v>
       </c>
       <c r="N33" s="5" t="inlineStr">
         <is>
-          <t>Moscow Textile</t>
+          <t>Xitoy Import</t>
         </is>
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P33" s="7" t="inlineStr">
@@ -2708,12 +2708,12 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>KK-1027</t>
+          <t>MS-1030</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>H&amp;M Qishki kurtka Sariq</t>
+          <t>Erkaklar to'q ko'k vitrofka</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -2723,54 +2723,54 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>H&amp;M</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>XXL</t>
+          <t>52, 54, 56</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>Sariq</t>
+          <t>to'q ko'k</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>Ayol</t>
+          <t>Erkak</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Polyester</t>
+          <t>Plashovka</t>
         </is>
       </c>
       <c r="J34" s="6" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="K34" s="6" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>1170391</v>
+        <v>90000</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>2066000</v>
+        <v>140000</v>
       </c>
       <c r="N34" s="5" t="inlineStr">
         <is>
-          <t>Istanbul Textile Co</t>
+          <t>Xitoy Import</t>
         </is>
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>11.04.2026</t>
-        </is>
-      </c>
-      <c r="P34" s="9" t="inlineStr">
-        <is>
-          <t>Tugagan</t>
+          <t>04.10.2026</t>
+        </is>
+      </c>
+      <c r="P34" s="7" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
         </is>
       </c>
     </row>
@@ -2780,12 +2780,12 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>KK-1028</t>
+          <t>MS-1031</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Zara Yengil kurtka Bordo</t>
+          <t>Yosh bolalar Boss vitrofka</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -2795,54 +2795,54 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Zara</t>
+          <t>Boss</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>Standart, 5-8 yosh</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>Bordo</t>
+          <t>to'q ko'k</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>Erkak</t>
+          <t>Bolalar</t>
         </is>
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Paxta + Polyester</t>
+          <t>Plashovka</t>
         </is>
       </c>
       <c r="J35" s="6" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="K35" s="6" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="L35" s="6" t="n">
-        <v>716643</v>
+        <v>55000</v>
       </c>
       <c r="M35" s="6" t="n">
-        <v>1040000</v>
+        <v>85000</v>
       </c>
       <c r="N35" s="5" t="inlineStr">
         <is>
-          <t>Local Factory UZ</t>
+          <t>Guangzhou Baby</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>02.08.2026</t>
-        </is>
-      </c>
-      <c r="P35" s="8" t="inlineStr">
-        <is>
-          <t>Kam qolgan</t>
+          <t>04.10.2026</t>
+        </is>
+      </c>
+      <c r="P35" s="7" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
         </is>
       </c>
     </row>
@@ -2852,69 +2852,69 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>KK-1042</t>
+          <t>MS-1032</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Adidas Yengil palto Moviy</t>
+          <t>Bolalar jinsi troyka komplekt</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Palto</t>
+          <t>Kostyum</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>XL</t>
+          <t>90, 100, 110</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>Moviy</t>
+          <t>bej, ko'k</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>Erkak</t>
+          <t>Bolalar</t>
         </is>
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Jun</t>
+          <t>Jinsi + paxta</t>
         </is>
       </c>
       <c r="J36" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K36" s="6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>1395038</v>
+        <v>110000</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>2041000</v>
+        <v>170000</v>
       </c>
       <c r="N36" s="5" t="inlineStr">
         <is>
-          <t>Local Factory UZ</t>
+          <t>Turkiya Baby</t>
         </is>
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>08.07.2026</t>
-        </is>
-      </c>
-      <c r="P36" s="8" t="inlineStr">
-        <is>
-          <t>Kam qolgan</t>
+          <t>04.10.2026</t>
+        </is>
+      </c>
+      <c r="P36" s="7" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
         </is>
       </c>
     </row>
@@ -2924,64 +2924,64 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>KK-1044</t>
+          <t>MS-1033</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Artel Style Klassik palto Ko'k</t>
+          <t>Yosh bolalar Polo vitrofka</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Palto</t>
+          <t>Kurtka</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>Artel Style</t>
+          <t>Polo</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>130, 140, 150, 160, 170</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>Ko'k</t>
+          <t>to'q ko'k</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>Ayol</t>
+          <t>Bolalar</t>
         </is>
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Jun</t>
+          <t>Plashovka</t>
         </is>
       </c>
       <c r="J37" s="6" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K37" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>1782729</v>
+        <v>62000</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>3162000</v>
+        <v>95000</v>
       </c>
       <c r="N37" s="5" t="inlineStr">
         <is>
-          <t>Local Factory UZ</t>
+          <t>Guangzhou Baby</t>
         </is>
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>26.07.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P37" s="7" t="inlineStr">
@@ -2996,64 +2996,64 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>KK-1043</t>
+          <t>MS-1034</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Artel Style Uzun palto Qizil</t>
+          <t>Erkaklar AQSh bayroqli svitir</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Palto</t>
+          <t>Svitir</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>Artel Style</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>XL</t>
+          <t>L, XL, XXL</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>Qizil</t>
+          <t>xaki, zaytun</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>Bolalar</t>
+          <t>Erkak</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Polyester</t>
+          <t>Paxta trikotaj</t>
         </is>
       </c>
       <c r="J38" s="6" t="n">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="K38" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>1333920</v>
+        <v>45000</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>1883000</v>
+        <v>70000</v>
       </c>
       <c r="N38" s="5" t="inlineStr">
         <is>
-          <t>Toshkent Optom</t>
+          <t>Toshkent Tekstil</t>
         </is>
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>16.04.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P38" s="7" t="inlineStr">
@@ -3068,64 +3068,64 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>KK-1047</t>
+          <t>MS-1035</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Koton Klassik palto Qora</t>
+          <t>Erkaklar kapyushonli xudi svitir</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Palto</t>
+          <t>Svitir</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>Koton</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>L, XL, XXL</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>Qora</t>
+          <t>kulrang</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>Bolalar</t>
+          <t>Erkak</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Polyester</t>
+          <t>Qalin trikotaj</t>
         </is>
       </c>
       <c r="J39" s="6" t="n">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="K39" s="6" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>920845</v>
+        <v>55000</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>1397000</v>
+        <v>85000</v>
       </c>
       <c r="N39" s="5" t="inlineStr">
         <is>
-          <t>Moscow Textile</t>
+          <t>Toshkent Tekstil</t>
         </is>
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>19.05.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P39" s="7" t="inlineStr">
@@ -3140,64 +3140,64 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>KK-1046</t>
+          <t>MS-1036</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Local Brand UZ Yengil palto Oq</t>
+          <t>Erkaklar kulrang sportivka kostyum</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Palto</t>
+          <t>Kostyum</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Local Brand UZ</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L, XL, XXL</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>Oq</t>
+          <t>kulrang</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>Uniseks</t>
+          <t>Erkak</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Cashmere blend</t>
+          <t>Sifatli ikki ipli trikotaj</t>
         </is>
       </c>
       <c r="J40" s="6" t="n">
-        <v>76</v>
+        <v>7</v>
       </c>
       <c r="K40" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L40" s="6" t="n">
-        <v>1328139</v>
+        <v>140000</v>
       </c>
       <c r="M40" s="6" t="n">
-        <v>2080000</v>
+        <v>210000</v>
       </c>
       <c r="N40" s="5" t="inlineStr">
         <is>
-          <t>Moscow Textile</t>
+          <t>Turkiya Import</t>
         </is>
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>27.06.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P40" s="7" t="inlineStr">
@@ -3212,69 +3212,69 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>KK-1049</t>
+          <t>MS-1037</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Pull&amp;Bear Yengil palto Yashil</t>
+          <t>Ayollar dvoyka ko'ylak-yubka komplekt</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Palto</t>
+          <t>Ko'ylak</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>Pull&amp;Bear</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>XL</t>
+          <t>48, 50, 52, 54</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>Yashil</t>
+          <t>bordo, qora, kulrang</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>Erkak</t>
+          <t>Ayol</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Polyester</t>
+          <t>Trikotaj va jakkard</t>
         </is>
       </c>
       <c r="J41" s="6" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="K41" s="6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L41" s="6" t="n">
-        <v>1313742</v>
+        <v>145000</v>
       </c>
       <c r="M41" s="6" t="n">
-        <v>1891000</v>
+        <v>220000</v>
       </c>
       <c r="N41" s="5" t="inlineStr">
         <is>
-          <t>Dubai Fashion Hub</t>
+          <t>Samarqand Tekstil</t>
         </is>
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>21.07.2026</t>
-        </is>
-      </c>
-      <c r="P41" s="8" t="inlineStr">
-        <is>
-          <t>Kam qolgan</t>
+          <t>04.10.2026</t>
+        </is>
+      </c>
+      <c r="P41" s="7" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
         </is>
       </c>
     </row>
@@ -3284,69 +3284,69 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>KK-1045</t>
+          <t>MS-1038</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Puma Uzun palto Kulrang</t>
+          <t>Qiz bolalar uchun pijama komplekt</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Palto</t>
+          <t>Pijama</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>Puma</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Standart, 4-7 yosh</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>Kulrang</t>
+          <t>siyohrang, sariq, mentol</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>Uniseks</t>
+          <t>Bolalar</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Jun</t>
+          <t>Paxta 100%</t>
         </is>
       </c>
       <c r="J42" s="6" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="K42" s="6" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="L42" s="6" t="n">
-        <v>1431844</v>
+        <v>15000</v>
       </c>
       <c r="M42" s="6" t="n">
-        <v>2535000</v>
+        <v>25000</v>
       </c>
       <c r="N42" s="5" t="inlineStr">
         <is>
-          <t>Istanbul Import</t>
+          <t>Namangan Tekstil</t>
         </is>
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
-          <t>10.09.2026</t>
-        </is>
-      </c>
-      <c r="P42" s="8" t="inlineStr">
-        <is>
-          <t>Kam qolgan</t>
+          <t>04.10.2026</t>
+        </is>
+      </c>
+      <c r="P42" s="7" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
         </is>
       </c>
     </row>
@@ -3356,32 +3356,32 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>KK-1048</t>
+          <t>MS-1039</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Zara Yengil palto Bej</t>
+          <t>O'g'il bolalar uchun pijama komplekt</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Palto</t>
+          <t>Pijama</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>Zara</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>XL</t>
+          <t>Standart, 4-7 yosh</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>Bej</t>
+          <t>havorang, qora, yashil</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
@@ -3391,29 +3391,29 @@
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>Cashmere blend</t>
+          <t>Paxta 100%</t>
         </is>
       </c>
       <c r="J43" s="6" t="n">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="K43" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L43" s="6" t="n">
-        <v>1184954</v>
+        <v>18000</v>
       </c>
       <c r="M43" s="6" t="n">
-        <v>2062000</v>
+        <v>30000</v>
       </c>
       <c r="N43" s="5" t="inlineStr">
         <is>
-          <t>Istanbul Import</t>
+          <t>Namangan Tekstil</t>
         </is>
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
-          <t>03.06.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P43" s="7" t="inlineStr">
@@ -3428,32 +3428,32 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>KK-1069</t>
+          <t>MS-1040</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Adidas Ko'rinmas paypoq Bordo</t>
+          <t>O'g'il bolalar Xitoy krossovka</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Paypoq</t>
+          <t>Oyoq kiyim</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>43-46</t>
+          <t>26, 27, 28, 29, 30</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>Bordo</t>
+          <t>qora-oq</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
@@ -3463,29 +3463,29 @@
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Synthetics</t>
+          <t>To'qima mato va rezina</t>
         </is>
       </c>
       <c r="J44" s="6" t="n">
-        <v>68</v>
+        <v>12</v>
       </c>
       <c r="K44" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L44" s="6" t="n">
-        <v>57461</v>
+        <v>48000</v>
       </c>
       <c r="M44" s="6" t="n">
-        <v>102000</v>
+        <v>75000</v>
       </c>
       <c r="N44" s="5" t="inlineStr">
         <is>
-          <t>Istanbul Import</t>
+          <t>Guangzhou Shoes</t>
         </is>
       </c>
       <c r="O44" s="4" t="inlineStr">
         <is>
-          <t>24.05.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="P44" s="7" t="inlineStr">
@@ -3500,643 +3500,67 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>KK-1065</t>
+          <t>MS-1041</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Adidas Oddiy paypoq Bordo</t>
+          <t>Qiz bolalar Xitoy krossovka</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Paypoq</t>
+          <t>Oyoq kiyim</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>MarkazSavdo</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>39-42</t>
+          <t>26, 27, 28, 29, 30, 31</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>Bordo</t>
+          <t>oq-binafsharang, pushti</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>Ayol</t>
+          <t>Bolalar</t>
         </is>
       </c>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>Jun</t>
+          <t>To'qima mato va yengil taglik</t>
         </is>
       </c>
       <c r="J45" s="6" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="K45" s="6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L45" s="6" t="n">
-        <v>32435</v>
+        <v>55000</v>
       </c>
       <c r="M45" s="6" t="n">
-        <v>49000</v>
+        <v>85000</v>
       </c>
       <c r="N45" s="5" t="inlineStr">
         <is>
-          <t>Toshkent Optom</t>
+          <t>Guangzhou Shoes</t>
         </is>
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
-          <t>17.04.2026</t>
-        </is>
-      </c>
-      <c r="P45" s="8" t="inlineStr">
-        <is>
-          <t>Kam qolgan</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="n">
-        <v>42</v>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>KK-1071</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>Bershka Ko'rinmas paypoq Yashil</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>Paypoq</t>
-        </is>
-      </c>
-      <c r="E46" s="4" t="inlineStr">
-        <is>
-          <t>Bershka</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>39-42</t>
-        </is>
-      </c>
-      <c r="G46" s="4" t="inlineStr">
-        <is>
-          <t>Yashil</t>
-        </is>
-      </c>
-      <c r="H46" s="4" t="inlineStr">
-        <is>
-          <t>Bolalar</t>
-        </is>
-      </c>
-      <c r="I46" s="4" t="inlineStr">
-        <is>
-          <t>Jun</t>
-        </is>
-      </c>
-      <c r="J46" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="K46" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L46" s="6" t="n">
-        <v>66363</v>
-      </c>
-      <c r="M46" s="6" t="n">
-        <v>108000</v>
-      </c>
-      <c r="N46" s="5" t="inlineStr">
-        <is>
-          <t>Guangzhou Trade</t>
-        </is>
-      </c>
-      <c r="O46" s="4" t="inlineStr">
-        <is>
-          <t>02.08.2026</t>
-        </is>
-      </c>
-      <c r="P46" s="7" t="inlineStr">
-        <is>
-          <t>Mavjud</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="n">
-        <v>43</v>
-      </c>
-      <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>KK-1066</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>Defacto Sport paypoq Jigarrang</t>
-        </is>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>Paypoq</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>Defacto</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>43-46</t>
-        </is>
-      </c>
-      <c r="G47" s="4" t="inlineStr">
-        <is>
-          <t>Jigarrang</t>
-        </is>
-      </c>
-      <c r="H47" s="4" t="inlineStr">
-        <is>
-          <t>Uniseks</t>
-        </is>
-      </c>
-      <c r="I47" s="4" t="inlineStr">
-        <is>
-          <t>Jun</t>
-        </is>
-      </c>
-      <c r="J47" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="K47" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="L47" s="6" t="n">
-        <v>50138</v>
-      </c>
-      <c r="M47" s="6" t="n">
-        <v>69000</v>
-      </c>
-      <c r="N47" s="5" t="inlineStr">
-        <is>
-          <t>Dubai Fashion Hub</t>
-        </is>
-      </c>
-      <c r="O47" s="4" t="inlineStr">
-        <is>
-          <t>22.05.2026</t>
-        </is>
-      </c>
-      <c r="P47" s="7" t="inlineStr">
-        <is>
-          <t>Mavjud</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="n">
-        <v>44</v>
-      </c>
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>KK-1068</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>Defacto Sport paypoq Yashil</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>Paypoq</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>Defacto</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>43-46</t>
-        </is>
-      </c>
-      <c r="G48" s="4" t="inlineStr">
-        <is>
-          <t>Yashil</t>
-        </is>
-      </c>
-      <c r="H48" s="4" t="inlineStr">
-        <is>
-          <t>Uniseks</t>
-        </is>
-      </c>
-      <c r="I48" s="4" t="inlineStr">
-        <is>
-          <t>Synthetics</t>
-        </is>
-      </c>
-      <c r="J48" s="6" t="n">
-        <v>55</v>
-      </c>
-      <c r="K48" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L48" s="6" t="n">
-        <v>70711</v>
-      </c>
-      <c r="M48" s="6" t="n">
-        <v>100000</v>
-      </c>
-      <c r="N48" s="5" t="inlineStr">
-        <is>
-          <t>Local Factory UZ</t>
-        </is>
-      </c>
-      <c r="O48" s="4" t="inlineStr">
-        <is>
-          <t>01.08.2026</t>
-        </is>
-      </c>
-      <c r="P48" s="7" t="inlineStr">
-        <is>
-          <t>Mavjud</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="n">
-        <v>45</v>
-      </c>
-      <c r="B49" s="4" t="inlineStr">
-        <is>
-          <t>KK-1070</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>UzTex Qishki paypoq Bej</t>
-        </is>
-      </c>
-      <c r="D49" s="4" t="inlineStr">
-        <is>
-          <t>Paypoq</t>
-        </is>
-      </c>
-      <c r="E49" s="4" t="inlineStr">
-        <is>
-          <t>UzTex</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>39-42</t>
-        </is>
-      </c>
-      <c r="G49" s="4" t="inlineStr">
-        <is>
-          <t>Bej</t>
-        </is>
-      </c>
-      <c r="H49" s="4" t="inlineStr">
-        <is>
-          <t>Erkak</t>
-        </is>
-      </c>
-      <c r="I49" s="4" t="inlineStr">
-        <is>
-          <t>Synthetics</t>
-        </is>
-      </c>
-      <c r="J49" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="K49" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="L49" s="6" t="n">
-        <v>29903</v>
-      </c>
-      <c r="M49" s="6" t="n">
-        <v>45000</v>
-      </c>
-      <c r="N49" s="5" t="inlineStr">
-        <is>
-          <t>Guangzhou Trade</t>
-        </is>
-      </c>
-      <c r="O49" s="4" t="inlineStr">
-        <is>
-          <t>05.07.2026</t>
-        </is>
-      </c>
-      <c r="P49" s="8" t="inlineStr">
-        <is>
-          <t>Kam qolgan</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="n">
-        <v>46</v>
-      </c>
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>KK-1067</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>UzTex Sport paypoq Qizil</t>
-        </is>
-      </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>Paypoq</t>
-        </is>
-      </c>
-      <c r="E50" s="4" t="inlineStr">
-        <is>
-          <t>UzTex</t>
-        </is>
-      </c>
-      <c r="F50" s="4" t="inlineStr">
-        <is>
-          <t>39-42</t>
-        </is>
-      </c>
-      <c r="G50" s="4" t="inlineStr">
-        <is>
-          <t>Qizil</t>
-        </is>
-      </c>
-      <c r="H50" s="4" t="inlineStr">
-        <is>
-          <t>Bolalar</t>
-        </is>
-      </c>
-      <c r="I50" s="4" t="inlineStr">
-        <is>
-          <t>Jun</t>
-        </is>
-      </c>
-      <c r="J50" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K50" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="L50" s="6" t="n">
-        <v>79884</v>
-      </c>
-      <c r="M50" s="6" t="n">
-        <v>127000</v>
-      </c>
-      <c r="N50" s="5" t="inlineStr">
-        <is>
-          <t>Moscow Textile</t>
-        </is>
-      </c>
-      <c r="O50" s="4" t="inlineStr">
-        <is>
-          <t>27.05.2026</t>
-        </is>
-      </c>
-      <c r="P50" s="9" t="inlineStr">
-        <is>
-          <t>Tugagan</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="n">
-        <v>47</v>
-      </c>
-      <c r="B51" s="4" t="inlineStr">
-        <is>
-          <t>KK-1017</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>Artel Style Cargo shim Oq</t>
-        </is>
-      </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>Shim</t>
-        </is>
-      </c>
-      <c r="E51" s="4" t="inlineStr">
-        <is>
-          <t>Artel Style</t>
-        </is>
-      </c>
-      <c r="F51" s="4" t="inlineStr">
-        <is>
-          <t>36</t>
-        </is>
-      </c>
-      <c r="G51" s="4" t="inlineStr">
-        <is>
-          <t>Oq</t>
-        </is>
-      </c>
-      <c r="H51" s="4" t="inlineStr">
-        <is>
-          <t>Erkak</t>
-        </is>
-      </c>
-      <c r="I51" s="4" t="inlineStr">
-        <is>
-          <t>Polyester</t>
-        </is>
-      </c>
-      <c r="J51" s="6" t="n">
-        <v>31</v>
-      </c>
-      <c r="K51" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L51" s="6" t="n">
-        <v>267194</v>
-      </c>
-      <c r="M51" s="6" t="n">
-        <v>401000</v>
-      </c>
-      <c r="N51" s="5" t="inlineStr">
-        <is>
-          <t>Local Factory UZ</t>
-        </is>
-      </c>
-      <c r="O51" s="4" t="inlineStr">
-        <is>
-          <t>06.08.2026</t>
-        </is>
-      </c>
-      <c r="P51" s="7" t="inlineStr">
-        <is>
-          <t>Mavjud</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="4" t="n">
-        <v>48</v>
-      </c>
-      <c r="B52" s="4" t="inlineStr">
-        <is>
-          <t>KK-1013</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>Defacto Chino shim Bej</t>
-        </is>
-      </c>
-      <c r="D52" s="4" t="inlineStr">
-        <is>
-          <t>Shim</t>
-        </is>
-      </c>
-      <c r="E52" s="4" t="inlineStr">
-        <is>
-          <t>Defacto</t>
-        </is>
-      </c>
-      <c r="F52" s="4" t="inlineStr">
-        <is>
-          <t>36</t>
-        </is>
-      </c>
-      <c r="G52" s="4" t="inlineStr">
-        <is>
-          <t>Bej</t>
-        </is>
-      </c>
-      <c r="H52" s="4" t="inlineStr">
-        <is>
-          <t>Erkak</t>
-        </is>
-      </c>
-      <c r="I52" s="4" t="inlineStr">
-        <is>
-          <t>Denim</t>
-        </is>
-      </c>
-      <c r="J52" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K52" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L52" s="6" t="n">
-        <v>488512</v>
-      </c>
-      <c r="M52" s="6" t="n">
-        <v>688000</v>
-      </c>
-      <c r="N52" s="5" t="inlineStr">
-        <is>
-          <t>Toshkent Optom</t>
-        </is>
-      </c>
-      <c r="O52" s="4" t="inlineStr">
-        <is>
-          <t>21.04.2026</t>
-        </is>
-      </c>
-      <c r="P52" s="9" t="inlineStr">
-        <is>
-          <t>Tugagan</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="4" t="n">
-        <v>49</v>
-      </c>
-      <c r="B53" s="4" t="inlineStr">
-        <is>
-          <t>KK-1016</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>LC Waikiki Klassik shim Yashil</t>
-        </is>
-      </c>
-      <c r="D53" s="4" t="inlineStr">
-        <is>
-          <t>Shim</t>
-        </is>
-      </c>
-      <c r="E53" s="4" t="inlineStr">
-        <is>
-          <t>LC Waikiki</t>
-        </is>
-      </c>
-      <c r="F53" s="4" t="inlineStr">
-        <is>
-          <t>38</t>
-        </is>
-      </c>
-      <c r="G53" s="4" t="inlineStr">
-        <is>
-          <t>Yashil</t>
-        </is>
-      </c>
-      <c r="H53" s="4" t="inlineStr">
-        <is>
-          <t>Erkak</t>
-        </is>
-      </c>
-      <c r="I53" s="4" t="inlineStr">
-        <is>
-          <t>Denim</t>
-        </is>
-      </c>
-      <c r="J53" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="K53" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="L53" s="6" t="n">
-        <v>276200</v>
-      </c>
-      <c r="M53" s="6" t="n">
-        <v>397000</v>
-      </c>
-      <c r="N53" s="5" t="inlineStr">
-        <is>
-          <t>Istanbul Import</t>
-        </is>
-      </c>
-      <c r="O53" s="4" t="inlineStr">
-        <is>
-          <t>10.09.2026</t>
-        </is>
-      </c>
-      <c r="P53" s="7" t="inlineStr">
+          <t>04.10.2026</t>
+        </is>
+      </c>
+      <c r="P45" s="7" t="inlineStr">
         <is>
           <t>Mavjud</t>
         </is>

</xml_diff>

<commit_message>
feat: world-class flagship upgrade v6.0 with @markazsavdo channel sync, VIP loyalty cashback, AI stylist, and abandoned order recovery
</commit_message>
<xml_diff>
--- a/reports/KIYIM_KECHAK_DOKONI_OMBOR_HISOBOTI.xlsx
+++ b/reports/KIYIM_KECHAK_DOKONI_OMBOR_HISOBOTI.xlsx
@@ -499,7 +499,7 @@
   <dimension ref="A1:P45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="86" customWidth="1" min="1" max="1"/>
+    <col width="84" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
@@ -527,7 +527,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Yaratilgan sana: 05.10.2026 | Kanal: @markazsavdo_7 | Do'kon egasi: Mansur Radjabov</t>
+          <t>Yaratilgan sana: 05.10.2026 | Kanal: @markazsavdo | Do'kon egasi: Mansur Radjabov</t>
         </is>
       </c>
     </row>

</xml_diff>